<commit_message>
Task 7 and report
</commit_message>
<xml_diff>
--- a/Statistics.xlsx
+++ b/Statistics.xlsx
@@ -8,12 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chris\Documents\ETS\Cours\LOG430-ArchitectureLog\Lab\4\log430-la4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C5A4B3F8-0600-4320-B065-D0A550160246}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E118BD44-805F-4DE6-AEAB-42133E03D19A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{89BBF7AC-0B90-40E5-B1A3-7302ED503753}"/>
+    <workbookView minimized="1" xWindow="-12" yWindow="6828" windowWidth="23064" windowHeight="6864" activeTab="2" xr2:uid="{89BBF7AC-0B90-40E5-B1A3-7302ED503753}"/>
+    <workbookView xWindow="-96" yWindow="6840" windowWidth="23232" windowHeight="6936" activeTab="2" xr2:uid="{B9D12060-3BF5-4A95-BA8F-4F5E63C26567}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="23232" windowHeight="6936" activeTab="1" xr2:uid="{D8E57206-AE9D-41E1-9755-9CEE91DCD051}"/>
   </bookViews>
   <sheets>
-    <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
+    <sheet name="Initial" sheetId="1" r:id="rId1"/>
+    <sheet name="Post add_order opt" sheetId="2" r:id="rId2"/>
+    <sheet name="Post Redis Optimisation" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="55">
   <si>
     <t>Type</t>
   </si>
@@ -123,19 +127,110 @@
   </si>
   <si>
     <t>652.18</t>
+  </si>
+  <si>
+    <t>8259.18</t>
+  </si>
+  <si>
+    <t>109.6</t>
+  </si>
+  <si>
+    <t>20.9</t>
+  </si>
+  <si>
+    <t>175.75</t>
+  </si>
+  <si>
+    <t>1049.12</t>
+  </si>
+  <si>
+    <t>19.5</t>
+  </si>
+  <si>
+    <t>117.47</t>
+  </si>
+  <si>
+    <t>297.56</t>
+  </si>
+  <si>
+    <t>17.9</t>
+  </si>
+  <si>
+    <t>17.6</t>
+  </si>
+  <si>
+    <t>2919.93</t>
+  </si>
+  <si>
+    <t>484.25</t>
+  </si>
+  <si>
+    <t>58.3</t>
+  </si>
+  <si>
+    <t>57.5</t>
+  </si>
+  <si>
+    <t>Taux erreurs requetes</t>
+  </si>
+  <si>
+    <t>12150.98</t>
+  </si>
+  <si>
+    <t>35.13</t>
+  </si>
+  <si>
+    <t>7.7</t>
+  </si>
+  <si>
+    <t>3061.69</t>
+  </si>
+  <si>
+    <t>309.84</t>
+  </si>
+  <si>
+    <t>5.9</t>
+  </si>
+  <si>
+    <t>3140.4</t>
+  </si>
+  <si>
+    <t>322.6</t>
+  </si>
+  <si>
+    <t>4.2</t>
+  </si>
+  <si>
+    <t>6535.64</t>
+  </si>
+  <si>
+    <t>209.34</t>
+  </si>
+  <si>
+    <t>17.8</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">
@@ -152,7 +247,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -160,13 +255,55 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF515151"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="FF515151"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -501,7 +638,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E05F804-BC31-4D65-B1CA-16455D76D1E3}">
-  <dimension ref="A1:M5"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
@@ -706,7 +843,528 @@
         <v>17</v>
       </c>
     </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B6" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6">
+        <f>D2/C2</f>
+        <v>0.98891352549889133</v>
+      </c>
+      <c r="D6" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(C6)</f>
+        <v>=D2/C2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B7" s="3"/>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B6:B7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1D4B368A-938B-4F0F-9B1B-997AE65079E1}">
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="28.21875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.6640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" s="9" customFormat="1" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="8" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2">
+        <v>819</v>
+      </c>
+      <c r="D2">
+        <v>813</v>
+      </c>
+      <c r="E2">
+        <v>13</v>
+      </c>
+      <c r="F2">
+        <v>60000</v>
+      </c>
+      <c r="G2">
+        <v>60000</v>
+      </c>
+      <c r="H2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>60020</v>
+      </c>
+      <c r="K2" t="s">
+        <v>29</v>
+      </c>
+      <c r="L2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3">
+        <v>800</v>
+      </c>
+      <c r="D3">
+        <v>627</v>
+      </c>
+      <c r="E3">
+        <v>61</v>
+      </c>
+      <c r="F3">
+        <v>470</v>
+      </c>
+      <c r="G3">
+        <v>870</v>
+      </c>
+      <c r="H3" t="s">
+        <v>31</v>
+      </c>
+      <c r="I3">
+        <v>12</v>
+      </c>
+      <c r="J3">
+        <v>1013</v>
+      </c>
+      <c r="K3" t="s">
+        <v>32</v>
+      </c>
+      <c r="L3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4">
+        <v>777</v>
+      </c>
+      <c r="D4">
+        <v>613</v>
+      </c>
+      <c r="E4">
+        <v>64</v>
+      </c>
+      <c r="F4">
+        <v>430</v>
+      </c>
+      <c r="G4">
+        <v>610</v>
+      </c>
+      <c r="H4" t="s">
+        <v>34</v>
+      </c>
+      <c r="I4">
+        <v>11</v>
+      </c>
+      <c r="J4">
+        <v>994</v>
+      </c>
+      <c r="K4" t="s">
+        <v>35</v>
+      </c>
+      <c r="L4" t="s">
+        <v>36</v>
+      </c>
+      <c r="M4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5">
+        <v>2396</v>
+      </c>
+      <c r="D5">
+        <v>2053</v>
+      </c>
+      <c r="E5">
+        <v>29</v>
+      </c>
+      <c r="F5">
+        <v>1000</v>
+      </c>
+      <c r="G5">
+        <v>60000</v>
+      </c>
+      <c r="H5" t="s">
+        <v>38</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>60020</v>
+      </c>
+      <c r="K5" t="s">
+        <v>39</v>
+      </c>
+      <c r="L5" t="s">
+        <v>40</v>
+      </c>
+      <c r="M5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B6" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6">
+        <f>D2/C2</f>
+        <v>0.9926739926739927</v>
+      </c>
+      <c r="D6" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(C6)</f>
+        <v>=D2/C2</v>
+      </c>
+      <c r="E6">
+        <f>D3/C3</f>
+        <v>0.78374999999999995</v>
+      </c>
+      <c r="F6" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(E6)</f>
+        <v>=D3/C3</v>
+      </c>
+      <c r="G6">
+        <f>D4/C4</f>
+        <v>0.78893178893178895</v>
+      </c>
+      <c r="H6" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(G6)</f>
+        <v>=D4/C4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B7" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B6:B7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71EC9DEE-568F-44B5-BD42-176642209527}">
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="28.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" ht="27" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="4">
+        <v>492</v>
+      </c>
+      <c r="D2" s="4">
+        <v>488</v>
+      </c>
+      <c r="E2" s="4">
+        <v>590</v>
+      </c>
+      <c r="F2" s="4">
+        <v>60000</v>
+      </c>
+      <c r="G2" s="4">
+        <v>60000</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="I2" s="4">
+        <v>0</v>
+      </c>
+      <c r="J2" s="4">
+        <v>60009</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="4">
+        <v>419</v>
+      </c>
+      <c r="D3" s="4">
+        <v>265</v>
+      </c>
+      <c r="E3" s="4">
+        <v>3200</v>
+      </c>
+      <c r="F3" s="4">
+        <v>7300</v>
+      </c>
+      <c r="G3" s="4">
+        <v>7600</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="I3" s="4">
+        <v>4</v>
+      </c>
+      <c r="J3" s="4">
+        <v>7693</v>
+      </c>
+      <c r="K3" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="4">
+        <v>385</v>
+      </c>
+      <c r="D4" s="4">
+        <v>241</v>
+      </c>
+      <c r="E4" s="4">
+        <v>3400</v>
+      </c>
+      <c r="F4" s="4">
+        <v>7300</v>
+      </c>
+      <c r="G4" s="4">
+        <v>7600</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="I4" s="4">
+        <v>4</v>
+      </c>
+      <c r="J4" s="4">
+        <v>7671</v>
+      </c>
+      <c r="K4" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="M4" s="4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="4">
+        <v>1296</v>
+      </c>
+      <c r="D5" s="4">
+        <v>994</v>
+      </c>
+      <c r="E5" s="4">
+        <v>790</v>
+      </c>
+      <c r="F5" s="4">
+        <v>60000</v>
+      </c>
+      <c r="G5" s="4">
+        <v>60000</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="I5" s="4">
+        <v>0</v>
+      </c>
+      <c r="J5" s="4">
+        <v>60009</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="M5" s="4" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B6" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6">
+        <f>D2/C2</f>
+        <v>0.99186991869918695</v>
+      </c>
+      <c r="D6" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(C6)</f>
+        <v>=D2/C2</v>
+      </c>
+      <c r="E6">
+        <f>D3/C3</f>
+        <v>0.63245823389021483</v>
+      </c>
+      <c r="F6" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(E6)</f>
+        <v>=D3/C3</v>
+      </c>
+      <c r="G6">
+        <f>D4/C4</f>
+        <v>0.62597402597402596</v>
+      </c>
+      <c r="H6" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(G6)</f>
+        <v>=D4/C4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B7" s="3"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B6:B7"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CD mods. Final TODO : Report
</commit_message>
<xml_diff>
--- a/Statistics.xlsx
+++ b/Statistics.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chris\Documents\ETS\Cours\LOG430-ArchitectureLog\Lab\4\log430-la4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E118BD44-805F-4DE6-AEAB-42133E03D19A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07765614-FA2A-44AD-96AE-643F2F0ADF88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView minimized="1" xWindow="-12" yWindow="6828" windowWidth="23064" windowHeight="6864" activeTab="2" xr2:uid="{89BBF7AC-0B90-40E5-B1A3-7302ED503753}"/>
     <workbookView xWindow="-96" yWindow="6840" windowWidth="23232" windowHeight="6936" activeTab="2" xr2:uid="{B9D12060-3BF5-4A95-BA8F-4F5E63C26567}"/>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="23232" windowHeight="6936" activeTab="1" xr2:uid="{D8E57206-AE9D-41E1-9755-9CEE91DCD051}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="23232" windowHeight="6936" activeTab="3" xr2:uid="{D8E57206-AE9D-41E1-9755-9CEE91DCD051}"/>
   </bookViews>
   <sheets>
     <sheet name="Initial" sheetId="1" r:id="rId1"/>
     <sheet name="Post add_order opt" sheetId="2" r:id="rId2"/>
     <sheet name="Post Redis Optimisation" sheetId="3" r:id="rId3"/>
+    <sheet name="Final" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="60">
   <si>
     <t>Type</t>
   </si>
@@ -208,6 +209,21 @@
   </si>
   <si>
     <t>17.8</t>
+  </si>
+  <si>
+    <t>0.33</t>
+  </si>
+  <si>
+    <t>0.28</t>
+  </si>
+  <si>
+    <t>1.5</t>
+  </si>
+  <si>
+    <t>0.26</t>
+  </si>
+  <si>
+    <t>2.5</t>
   </si>
 </sst>
 </file>
@@ -277,7 +293,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -303,6 +319,16 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1367,4 +1393,255 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7421EEF0-F559-4CAB-9A48-7767D242F7B8}">
+  <dimension ref="A1:M7"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="28.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:13" s="11" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="10" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="10" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="10" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="10" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" s="10" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="10" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="4">
+        <v>22</v>
+      </c>
+      <c r="D2" s="4">
+        <v>22</v>
+      </c>
+      <c r="E2" s="4">
+        <v>0</v>
+      </c>
+      <c r="F2" s="4">
+        <v>1</v>
+      </c>
+      <c r="G2" s="4">
+        <v>1</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="I2" s="4">
+        <v>0</v>
+      </c>
+      <c r="J2" s="4">
+        <v>1</v>
+      </c>
+      <c r="K2" s="4">
+        <v>0</v>
+      </c>
+      <c r="L2" s="4">
+        <v>3</v>
+      </c>
+      <c r="M2" s="4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="4">
+        <v>28</v>
+      </c>
+      <c r="D3" s="4">
+        <v>28</v>
+      </c>
+      <c r="E3" s="4">
+        <v>0</v>
+      </c>
+      <c r="F3" s="4">
+        <v>1</v>
+      </c>
+      <c r="G3" s="4">
+        <v>1</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I3" s="4">
+        <v>0</v>
+      </c>
+      <c r="J3" s="4">
+        <v>1</v>
+      </c>
+      <c r="K3" s="4">
+        <v>0</v>
+      </c>
+      <c r="L3" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="4">
+        <v>32</v>
+      </c>
+      <c r="D4" s="4">
+        <v>32</v>
+      </c>
+      <c r="E4" s="4">
+        <v>0</v>
+      </c>
+      <c r="F4" s="4">
+        <v>1</v>
+      </c>
+      <c r="G4" s="4">
+        <v>1</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="I4" s="4">
+        <v>0</v>
+      </c>
+      <c r="J4" s="4">
+        <v>1</v>
+      </c>
+      <c r="K4" s="4">
+        <v>0</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="M4" s="4" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A5" s="4"/>
+      <c r="B5" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="4">
+        <v>82</v>
+      </c>
+      <c r="D5" s="4">
+        <v>82</v>
+      </c>
+      <c r="E5" s="4">
+        <v>0</v>
+      </c>
+      <c r="F5" s="4">
+        <v>1</v>
+      </c>
+      <c r="G5" s="4">
+        <v>1</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="I5" s="4">
+        <v>0</v>
+      </c>
+      <c r="J5" s="4">
+        <v>1</v>
+      </c>
+      <c r="K5" s="4">
+        <v>0</v>
+      </c>
+      <c r="L5" s="4">
+        <v>7</v>
+      </c>
+      <c r="M5" s="4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B6" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6">
+        <f>D2/C2</f>
+        <v>1</v>
+      </c>
+      <c r="D6" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(C6)</f>
+        <v>=D2/C2</v>
+      </c>
+      <c r="E6">
+        <f>D3/C3</f>
+        <v>1</v>
+      </c>
+      <c r="F6" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(E6)</f>
+        <v>=D3/C3</v>
+      </c>
+      <c r="G6">
+        <f>D4/C4</f>
+        <v>1</v>
+      </c>
+      <c r="H6" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(G6)</f>
+        <v>=D4/C4</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B7" s="13"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="B6:B7"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>